<commit_message>
Major updates: subcaption mapping, risk logic, pie colors, portfolio risk
- Hardcode complete ANSWER_SUBCAPTIONS lookup for all Q&A slides so every
  answer shows its correct italic subcaption (employment, income, liability,
  horizon, fall reaction)
- Add liability management step (step 4) to calc_risk_profile: 'Just about'
  or 'No - struggling' downgrades risk tier by 1
- Fix pie chart colors to match PowerUp_Base_Deck legend exactly:
  Debt=#EBF2F2, Gold=#F7CB88, Global=#FFC7B4, Solution=#CABAF3
- Add _portfolio_risk() — derives risk from S+M allocation thresholds
- Slide 4: show calculated portfolio risk, green/red match text vs questionnaire risk
- Slide 3: SIP step-up text box shown/removed based on YoY increase %; no * when 0
- Update data files (PF_level, Riskgroup, Scheme, Lines, Results, Invested)

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PowerUp Questionnaire Responses Sample.xlsx
+++ b/PowerUp Questionnaire Responses Sample.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\PowerUpInfinite\M2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CB6B08EC-9D76-4277-AA90-0D790131F8BB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FC05DF51-8719-44BB-99BE-DA64AD60D8FD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="116" uniqueCount="104">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="236" uniqueCount="169">
   <si>
     <t>Timestamp</t>
   </si>
@@ -333,6 +333,201 @@
   </si>
   <si>
     <t>MFUf5625b488dff44ca91d0d9650e2c1891</t>
+  </si>
+  <si>
+    <t>2026-03-28 19:47:02 IST</t>
+  </si>
+  <si>
+    <t>Chirag Gabani</t>
+  </si>
+  <si>
+    <t>patelchirag01@gmail.com</t>
+  </si>
+  <si>
+    <t>36-45</t>
+  </si>
+  <si>
+    <t>No Fixed Goal</t>
+  </si>
+  <si>
+    <t>More than 24 months</t>
+  </si>
+  <si>
+    <t>2026-03-31 17:47:22 IST</t>
+  </si>
+  <si>
+    <t>Kapil Pahwa</t>
+  </si>
+  <si>
+    <t>pahwakapil@gmail.com</t>
+  </si>
+  <si>
+    <t>Retirement Planning, Children Education, Children Marriage</t>
+  </si>
+  <si>
+    <t>7-12 months</t>
+  </si>
+  <si>
+    <t>RD 7L</t>
+  </si>
+  <si>
+    <t>9500000 ending in 2047</t>
+  </si>
+  <si>
+    <t>Saira Pahwa</t>
+  </si>
+  <si>
+    <t>16 years</t>
+  </si>
+  <si>
+    <t>Anaya Pahwa</t>
+  </si>
+  <si>
+    <t>22 years</t>
+  </si>
+  <si>
+    <t>2026-03-31 19:05:22 IST</t>
+  </si>
+  <si>
+    <t>CHAYKAM SRINIVASA REDDY</t>
+  </si>
+  <si>
+    <t>creddy422@gmail.com</t>
+  </si>
+  <si>
+    <t>56+</t>
+  </si>
+  <si>
+    <t>Retired</t>
+  </si>
+  <si>
+    <t>Passive Income Only</t>
+  </si>
+  <si>
+    <t>Post-Retirement Income Planning, Wealth Conservation, Children Marriage</t>
+  </si>
+  <si>
+    <t>FD 1 CR STOCKS 40L</t>
+  </si>
+  <si>
+    <t>FD 1CR STOCKS 40L</t>
+  </si>
+  <si>
+    <t>Lalasa</t>
+  </si>
+  <si>
+    <t>5 years</t>
+  </si>
+  <si>
+    <t>2026-03-31 21:04:53 IST</t>
+  </si>
+  <si>
+    <t>Azad</t>
+  </si>
+  <si>
+    <t>azad1472@gmail.com</t>
+  </si>
+  <si>
+    <t>Soon to be Retiring (within 5 yrs)</t>
+  </si>
+  <si>
+    <t>FD - 40L, Stocks - 30L</t>
+  </si>
+  <si>
+    <t>Home loan EMI - Monthly- 1.05L</t>
+  </si>
+  <si>
+    <t>Saahil Singh</t>
+  </si>
+  <si>
+    <t>5 - 6 years</t>
+  </si>
+  <si>
+    <t>Shaury Pratap Singh</t>
+  </si>
+  <si>
+    <t>9 - 10 years</t>
+  </si>
+  <si>
+    <t>2026-04-01 19:20:02 IST</t>
+  </si>
+  <si>
+    <t>Luv Kumar</t>
+  </si>
+  <si>
+    <t>luvkumar02@gmail.com</t>
+  </si>
+  <si>
+    <t>Passive + Pension Income</t>
+  </si>
+  <si>
+    <t>Wealth Conservation, Other</t>
+  </si>
+  <si>
+    <t>PPF 20 lac</t>
+  </si>
+  <si>
+    <t>2026-04-01 20:29:55 IST</t>
+  </si>
+  <si>
+    <t>Navin Jhanji</t>
+  </si>
+  <si>
+    <t>navin.jhanji@gmail.com</t>
+  </si>
+  <si>
+    <t>Dependent liabilities only</t>
+  </si>
+  <si>
+    <t>Just about</t>
+  </si>
+  <si>
+    <t>DJ1</t>
+  </si>
+  <si>
+    <t>DJ2</t>
+  </si>
+  <si>
+    <t>2026-04-02 12:39:22 IST</t>
+  </si>
+  <si>
+    <t>Arti Srivastava</t>
+  </si>
+  <si>
+    <t>arati.r.srivastava@gmail.com</t>
+  </si>
+  <si>
+    <t>Retirement Planning, Home Purchase, Children Education, Children Marriage</t>
+  </si>
+  <si>
+    <t>13-24 months</t>
+  </si>
+  <si>
+    <t>Nothing</t>
+  </si>
+  <si>
+    <t>Dhriti</t>
+  </si>
+  <si>
+    <t>20 years</t>
+  </si>
+  <si>
+    <t>Dont Know Yet</t>
+  </si>
+  <si>
+    <t>PF000015</t>
+  </si>
+  <si>
+    <t>MFU773a64e92fd641db81d6c47a7e820283</t>
+  </si>
+  <si>
+    <t>MFU7f2b0a924dde4979936c8a26db30ca3c</t>
+  </si>
+  <si>
+    <t>MFUd63f9f8f04964b468dd27771f31bb5a6</t>
+  </si>
+  <si>
+    <t>MFUc07b4b8fe26945d1a4eb998e296814ea</t>
   </si>
 </sst>
 </file>
@@ -1164,30 +1359,632 @@
       </c>
     </row>
     <row r="5" spans="1:67" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B5" s="3"/>
+      <c r="B5" s="3" t="s">
+        <v>104</v>
+      </c>
+      <c r="C5" t="s">
+        <v>105</v>
+      </c>
+      <c r="D5" t="s">
+        <v>106</v>
+      </c>
+      <c r="E5" t="s">
+        <v>107</v>
+      </c>
+      <c r="F5" t="s">
+        <v>70</v>
+      </c>
+      <c r="G5" t="s">
+        <v>84</v>
+      </c>
+      <c r="H5" t="s">
+        <v>108</v>
+      </c>
+      <c r="I5" t="s">
+        <v>73</v>
+      </c>
+      <c r="J5" t="s">
+        <v>74</v>
+      </c>
+      <c r="K5" t="s">
+        <v>109</v>
+      </c>
+      <c r="L5" t="s">
+        <v>99</v>
+      </c>
+      <c r="M5" t="s">
+        <v>77</v>
+      </c>
+      <c r="N5" t="s">
+        <v>78</v>
+      </c>
+      <c r="O5">
+        <v>10000000</v>
+      </c>
+      <c r="P5">
+        <v>500000</v>
+      </c>
+      <c r="Q5">
+        <v>0</v>
+      </c>
       <c r="AM5" s="2"/>
     </row>
     <row r="6" spans="1:67" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B6" s="3"/>
+      <c r="A6" t="s">
+        <v>168</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>110</v>
+      </c>
+      <c r="C6" t="s">
+        <v>111</v>
+      </c>
+      <c r="D6" t="s">
+        <v>112</v>
+      </c>
+      <c r="E6" t="s">
+        <v>107</v>
+      </c>
+      <c r="F6" t="s">
+        <v>70</v>
+      </c>
+      <c r="G6" t="s">
+        <v>84</v>
+      </c>
+      <c r="H6" t="s">
+        <v>113</v>
+      </c>
+      <c r="I6" t="s">
+        <v>86</v>
+      </c>
+      <c r="J6" t="s">
+        <v>87</v>
+      </c>
+      <c r="K6" t="s">
+        <v>114</v>
+      </c>
+      <c r="L6" t="s">
+        <v>76</v>
+      </c>
+      <c r="M6" t="s">
+        <v>77</v>
+      </c>
+      <c r="N6" t="s">
+        <v>78</v>
+      </c>
+      <c r="O6">
+        <v>5000000</v>
+      </c>
+      <c r="P6">
+        <v>100000</v>
+      </c>
+      <c r="Q6">
+        <v>0</v>
+      </c>
+      <c r="R6" t="s">
+        <v>115</v>
+      </c>
+      <c r="S6">
+        <v>415000</v>
+      </c>
+      <c r="T6">
+        <v>200000</v>
+      </c>
+      <c r="U6" s="4">
+        <v>-0.2</v>
+      </c>
+      <c r="V6">
+        <v>75000</v>
+      </c>
+      <c r="W6" s="4">
+        <v>0.1</v>
+      </c>
+      <c r="X6" t="s">
+        <v>116</v>
+      </c>
       <c r="AM6" s="2"/>
+      <c r="AN6">
+        <v>2034</v>
+      </c>
+      <c r="AO6">
+        <v>10000000</v>
+      </c>
+      <c r="AP6">
+        <v>2026</v>
+      </c>
+      <c r="AQ6">
+        <v>0</v>
+      </c>
+      <c r="AR6">
+        <v>2040</v>
+      </c>
+      <c r="AS6">
+        <v>12500000</v>
+      </c>
+      <c r="AT6">
+        <v>2026</v>
+      </c>
+      <c r="AU6">
+        <v>0</v>
+      </c>
+      <c r="BD6" t="s">
+        <v>117</v>
+      </c>
+      <c r="BE6" t="s">
+        <v>118</v>
+      </c>
+      <c r="BF6">
+        <v>7000000</v>
+      </c>
+      <c r="BG6" t="s">
+        <v>119</v>
+      </c>
+      <c r="BH6" t="s">
+        <v>120</v>
+      </c>
+      <c r="BI6">
+        <v>7000000</v>
+      </c>
     </row>
     <row r="7" spans="1:67" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B7" s="3"/>
+      <c r="B7" s="3" t="s">
+        <v>121</v>
+      </c>
+      <c r="C7" t="s">
+        <v>122</v>
+      </c>
+      <c r="D7" t="s">
+        <v>123</v>
+      </c>
+      <c r="E7" t="s">
+        <v>124</v>
+      </c>
+      <c r="F7" t="s">
+        <v>125</v>
+      </c>
+      <c r="G7" t="s">
+        <v>126</v>
+      </c>
+      <c r="H7" t="s">
+        <v>127</v>
+      </c>
+      <c r="I7" t="s">
+        <v>86</v>
+      </c>
+      <c r="J7" t="s">
+        <v>87</v>
+      </c>
+      <c r="K7" t="s">
+        <v>114</v>
+      </c>
+      <c r="L7" t="s">
+        <v>99</v>
+      </c>
+      <c r="M7" t="s">
+        <v>100</v>
+      </c>
+      <c r="N7" t="s">
+        <v>88</v>
+      </c>
+      <c r="O7">
+        <v>2000000</v>
+      </c>
+      <c r="P7">
+        <v>5000</v>
+      </c>
+      <c r="Q7">
+        <v>0</v>
+      </c>
+      <c r="R7" t="s">
+        <v>128</v>
+      </c>
+      <c r="Y7">
+        <v>30000</v>
+      </c>
+      <c r="Z7">
+        <v>30000</v>
+      </c>
+      <c r="AA7">
+        <v>200000</v>
+      </c>
+      <c r="AB7" t="s">
+        <v>129</v>
+      </c>
       <c r="AM7" s="2"/>
+      <c r="BD7" t="s">
+        <v>130</v>
+      </c>
+      <c r="BE7" t="s">
+        <v>131</v>
+      </c>
+      <c r="BF7">
+        <v>10000000</v>
+      </c>
     </row>
     <row r="8" spans="1:67" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B8" s="3"/>
+      <c r="A8" t="s">
+        <v>166</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>132</v>
+      </c>
+      <c r="C8" t="s">
+        <v>133</v>
+      </c>
+      <c r="D8" t="s">
+        <v>134</v>
+      </c>
+      <c r="E8" t="s">
+        <v>83</v>
+      </c>
+      <c r="F8" t="s">
+        <v>135</v>
+      </c>
+      <c r="G8" t="s">
+        <v>84</v>
+      </c>
+      <c r="H8" t="s">
+        <v>113</v>
+      </c>
+      <c r="I8" t="s">
+        <v>86</v>
+      </c>
+      <c r="J8" t="s">
+        <v>87</v>
+      </c>
+      <c r="K8" t="s">
+        <v>114</v>
+      </c>
+      <c r="L8" t="s">
+        <v>99</v>
+      </c>
+      <c r="M8" t="s">
+        <v>100</v>
+      </c>
+      <c r="N8" t="s">
+        <v>78</v>
+      </c>
+      <c r="O8">
+        <v>500000</v>
+      </c>
+      <c r="P8">
+        <v>200000</v>
+      </c>
+      <c r="Q8">
+        <v>0</v>
+      </c>
+      <c r="R8" t="s">
+        <v>136</v>
+      </c>
+      <c r="S8">
+        <v>400000</v>
+      </c>
+      <c r="T8">
+        <v>100000</v>
+      </c>
+      <c r="U8" s="4">
+        <v>0</v>
+      </c>
+      <c r="V8">
+        <v>175000</v>
+      </c>
+      <c r="W8" s="4">
+        <v>0</v>
+      </c>
+      <c r="X8" t="s">
+        <v>137</v>
+      </c>
+      <c r="AN8">
+        <v>2028</v>
+      </c>
+      <c r="AO8">
+        <v>15</v>
+      </c>
+      <c r="AP8">
+        <v>2032</v>
+      </c>
+      <c r="AQ8">
+        <v>30</v>
+      </c>
+      <c r="BD8" t="s">
+        <v>138</v>
+      </c>
+      <c r="BE8" t="s">
+        <v>139</v>
+      </c>
+      <c r="BF8">
+        <v>30</v>
+      </c>
+      <c r="BG8" t="s">
+        <v>140</v>
+      </c>
+      <c r="BH8" t="s">
+        <v>141</v>
+      </c>
+      <c r="BI8">
+        <v>30</v>
+      </c>
     </row>
     <row r="9" spans="1:67" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B9" s="3"/>
+      <c r="A9" t="s">
+        <v>167</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>142</v>
+      </c>
+      <c r="C9" t="s">
+        <v>143</v>
+      </c>
+      <c r="D9" t="s">
+        <v>144</v>
+      </c>
+      <c r="E9" t="s">
+        <v>124</v>
+      </c>
+      <c r="F9" t="s">
+        <v>125</v>
+      </c>
+      <c r="G9" t="s">
+        <v>145</v>
+      </c>
+      <c r="H9" t="s">
+        <v>146</v>
+      </c>
+      <c r="I9" t="s">
+        <v>73</v>
+      </c>
+      <c r="J9" t="s">
+        <v>74</v>
+      </c>
+      <c r="K9" t="s">
+        <v>109</v>
+      </c>
+      <c r="L9" t="s">
+        <v>76</v>
+      </c>
+      <c r="M9" t="s">
+        <v>77</v>
+      </c>
+      <c r="N9" t="s">
+        <v>88</v>
+      </c>
+      <c r="O9">
+        <v>10000</v>
+      </c>
+      <c r="P9">
+        <v>100</v>
+      </c>
+      <c r="Q9">
+        <v>0</v>
+      </c>
+      <c r="R9" t="s">
+        <v>147</v>
+      </c>
       <c r="AM9" s="2"/>
     </row>
     <row r="10" spans="1:67" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B10" s="3"/>
+      <c r="A10" t="s">
+        <v>164</v>
+      </c>
+      <c r="B10" s="3" t="s">
+        <v>148</v>
+      </c>
+      <c r="C10" t="s">
+        <v>149</v>
+      </c>
+      <c r="D10" t="s">
+        <v>150</v>
+      </c>
+      <c r="E10" t="s">
+        <v>83</v>
+      </c>
+      <c r="F10" t="s">
+        <v>70</v>
+      </c>
+      <c r="G10" t="s">
+        <v>71</v>
+      </c>
+      <c r="H10" t="s">
+        <v>98</v>
+      </c>
+      <c r="I10" t="s">
+        <v>151</v>
+      </c>
+      <c r="J10" t="s">
+        <v>152</v>
+      </c>
+      <c r="K10" t="s">
+        <v>109</v>
+      </c>
+      <c r="L10" t="s">
+        <v>99</v>
+      </c>
+      <c r="M10" t="s">
+        <v>77</v>
+      </c>
+      <c r="N10" t="s">
+        <v>88</v>
+      </c>
+      <c r="O10">
+        <v>25000000</v>
+      </c>
+      <c r="P10">
+        <v>200000</v>
+      </c>
+      <c r="Q10">
+        <v>0</v>
+      </c>
+      <c r="R10">
+        <v>20000000</v>
+      </c>
+      <c r="S10">
+        <v>0</v>
+      </c>
+      <c r="T10">
+        <v>100000</v>
+      </c>
+      <c r="U10" s="4">
+        <v>0</v>
+      </c>
+      <c r="V10">
+        <v>174000</v>
+      </c>
+      <c r="W10" s="4">
+        <v>0</v>
+      </c>
       <c r="AH10" s="2"/>
+      <c r="BD10" t="s">
+        <v>153</v>
+      </c>
+      <c r="BE10">
+        <v>4</v>
+      </c>
+      <c r="BF10">
+        <v>6000000</v>
+      </c>
+      <c r="BG10" t="s">
+        <v>154</v>
+      </c>
+      <c r="BH10">
+        <v>7</v>
+      </c>
+      <c r="BI10">
+        <v>7000000</v>
+      </c>
     </row>
     <row r="11" spans="1:67" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B11" s="3"/>
+      <c r="A11" t="s">
+        <v>165</v>
+      </c>
+      <c r="B11" s="3" t="s">
+        <v>155</v>
+      </c>
+      <c r="C11" t="s">
+        <v>156</v>
+      </c>
+      <c r="D11" t="s">
+        <v>157</v>
+      </c>
+      <c r="E11" t="s">
+        <v>107</v>
+      </c>
+      <c r="F11" t="s">
+        <v>70</v>
+      </c>
+      <c r="G11" t="s">
+        <v>71</v>
+      </c>
+      <c r="H11" t="s">
+        <v>158</v>
+      </c>
+      <c r="I11" t="s">
+        <v>151</v>
+      </c>
+      <c r="J11" t="s">
+        <v>87</v>
+      </c>
+      <c r="K11" t="s">
+        <v>159</v>
+      </c>
+      <c r="L11" t="s">
+        <v>76</v>
+      </c>
+      <c r="M11" t="s">
+        <v>77</v>
+      </c>
+      <c r="N11" t="s">
+        <v>78</v>
+      </c>
+      <c r="O11">
+        <v>5000000</v>
+      </c>
+      <c r="P11">
+        <v>200000</v>
+      </c>
+      <c r="Q11">
+        <v>0</v>
+      </c>
+      <c r="R11">
+        <v>20000000</v>
+      </c>
+      <c r="S11">
+        <v>1100000</v>
+      </c>
+      <c r="T11">
+        <v>400000</v>
+      </c>
+      <c r="U11" s="4">
+        <v>-0.4</v>
+      </c>
+      <c r="V11">
+        <v>200000</v>
+      </c>
+      <c r="W11" s="4">
+        <v>0.2</v>
+      </c>
+      <c r="X11" t="s">
+        <v>160</v>
+      </c>
+      <c r="AH11">
+        <v>2035</v>
+      </c>
+      <c r="AI11">
+        <v>20000000</v>
+      </c>
+      <c r="AJ11">
+        <v>5</v>
+      </c>
+      <c r="AK11" t="s">
+        <v>79</v>
+      </c>
+      <c r="AL11" s="4">
+        <v>0.1</v>
+      </c>
+      <c r="AM11">
+        <v>90000</v>
+      </c>
+      <c r="AN11">
+        <v>2038</v>
+      </c>
+      <c r="AO11">
+        <v>2000000</v>
+      </c>
+      <c r="AP11">
+        <v>2042</v>
+      </c>
+      <c r="AQ11">
+        <v>7000000</v>
+      </c>
+      <c r="AR11">
+        <v>2057</v>
+      </c>
+      <c r="AS11">
+        <v>2000000</v>
+      </c>
+      <c r="AT11">
+        <v>2060</v>
+      </c>
+      <c r="AU11">
+        <v>15000000</v>
+      </c>
+      <c r="BD11" t="s">
+        <v>161</v>
+      </c>
+      <c r="BE11" t="s">
+        <v>162</v>
+      </c>
+      <c r="BF11">
+        <v>5000000</v>
+      </c>
+      <c r="BG11" t="s">
+        <v>163</v>
+      </c>
+      <c r="BH11">
+        <v>26</v>
+      </c>
+      <c r="BI11">
+        <v>5000000</v>
+      </c>
     </row>
     <row r="12" spans="1:67" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B12" s="3"/>

</xml_diff>